<commit_message>
chore: push current changes
</commit_message>
<xml_diff>
--- a/mock-report-output/failure-data.xlsx
+++ b/mock-report-output/failure-data.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="25" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="33" uniqueCount="29">
   <si>
     <t>Test ID</t>
   </si>
@@ -87,6 +87,21 @@
   </si>
   <si>
     <t>Increase timeout to 10s.</t>
+  </si>
+  <si>
+    <t>timeout-001</t>
+  </si>
+  <si>
+    <t>Search Module</t>
+  </si>
+  <si>
+    <t>Network Timeout during search initialization with a very long title to verify line clamping and responsiveness</t>
+  </si>
+  <si>
+    <t>timedOut</t>
+  </si>
+  <si>
+    <t>N/A</t>
   </si>
 </sst>
 </file>
@@ -477,7 +492,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="15" customWidth="1"/>
@@ -577,6 +592,35 @@
         <v>23</v>
       </c>
     </row>
+    <row r="4" spans="1:9" s="2" customFormat="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E4" s="2">
+        <v>30000</v>
+      </c>
+      <c r="F4" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G4" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="H4" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="I4" s="2" t="s">
+        <v>28</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967295" verticalDpi="4294967295" scale="100" fitToWidth="1" fitToHeight="1"/>

</xml_diff>